<commit_message>
some error check and fix
</commit_message>
<xml_diff>
--- a/Jay_Messages.xlsx
+++ b/Jay_Messages.xlsx
@@ -1,44 +1,77 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b6667756b8ce486a/Desktop/Maths game/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_4E3FA30D2C397D6A206102F4B86E91EBBF145690" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23E70C42-7FEE-43C7-997B-5436F9EC21EA}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Messages" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Date &amp; Time</t>
+  </si>
+  <si>
+    <t>Prediction Result</t>
+  </si>
+  <si>
+    <t>Message</t>
+  </si>
+  <si>
+    <t>2026-06-19 23:11:02</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-06-19 23:11:06</t>
+  </si>
+  <si>
+    <t>Thoda aur mehnat karo 📚</t>
+  </si>
+  <si>
+    <t>2026-06-19 23:11:03</t>
+  </si>
+  <si>
+    <t>2026-06-19 23:11:04</t>
+  </si>
+  <si>
+    <t>2026-06-19 23:11:07</t>
+  </si>
+  <si>
+    <t>2026-06-19 23:11:08</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -65,13 +98,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,166 +437,89 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="26.59765625" customWidth="1"/>
+    <col min="2" max="2" width="25.296875" customWidth="1"/>
+    <col min="3" max="3" width="33.09765625" customWidth="1"/>
+    <col min="4" max="4" width="34.69921875" customWidth="1"/>
+    <col min="5" max="5" width="31.59765625" customWidth="1"/>
+    <col min="6" max="6" width="23.59765625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Date &amp; Time</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Message</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Predicted Marks</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Prediction Result</v>
+    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
-        <v>2026-06-19 21:54:04</v>
-      </c>
-      <c r="C2" t="str">
-        <v>j</v>
-      </c>
-      <c r="D2" t="str">
-        <v>hi</v>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="str">
-        <v>2026-06-19 22:07:36</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Antigravity Test</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Hello from test suite!</v>
-      </c>
-      <c r="E3">
-        <v>95</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Topper ho kya? 🏆</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2026-06-19 22:10:27</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Antigravity Test</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Hello from test suite!</v>
-      </c>
-      <c r="E4">
-        <v>95</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Topper ho kya? 🏆</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2026-06-19 22:18:41</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Antigravity Test</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Hello from test suite!</v>
-      </c>
-      <c r="E5">
-        <v>95</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Topper ho kya? 🏆</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>2026-06-19 22:26:10</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Antigravity Test</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Hello from test suite!</v>
-      </c>
-      <c r="E6">
-        <v>95</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Topper ho kya? 🏆</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="str">
-        <v>2026-06-19 22:27:14</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Antigravity Test</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Hello from test suite!</v>
-      </c>
-      <c r="E7">
-        <v>95</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Topper ho kya? 🏆</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="str">
-        <v>2026-06-19 22:51:23</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Antigravity Test</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Hello from test suite!</v>
-      </c>
-      <c r="E8">
-        <v>95</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Topper ho kya? 🏆</v>
+      <c r="F3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError sqref="A1:B2 A3:B3 E1:F2 E3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>